<commit_message>
Moved IR to datapath
</commit_message>
<xml_diff>
--- a/ISA.xlsx
+++ b/ISA.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malco\CPUproj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4D37A37-DA0E-4FCB-AE9A-DC661A4B6B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A7EAE0-63CE-4B6E-BD7D-50AC16A1E5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Main" sheetId="1" r:id="rId1"/>
+    <sheet name="Control signals" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,9 +40,305 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
+  <si>
+    <t>Op Code</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>0011</t>
+  </si>
+  <si>
+    <t>0100</t>
+  </si>
+  <si>
+    <t>0101</t>
+  </si>
+  <si>
+    <t>0110</t>
+  </si>
+  <si>
+    <t>0111</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>1010</t>
+  </si>
+  <si>
+    <t>1011</t>
+  </si>
+  <si>
+    <t>1100</t>
+  </si>
+  <si>
+    <t>1101</t>
+  </si>
+  <si>
+    <t>1110</t>
+  </si>
+  <si>
+    <t>1111</t>
+  </si>
+  <si>
+    <t>Mnemonic</t>
+  </si>
+  <si>
+    <t>ADD</t>
+  </si>
+  <si>
+    <t>SUB</t>
+  </si>
+  <si>
+    <t>JMP</t>
+  </si>
+  <si>
+    <t>JTS</t>
+  </si>
+  <si>
+    <t>RET</t>
+  </si>
+  <si>
+    <t>LD</t>
+  </si>
+  <si>
+    <t>LDR</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>STR</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>OUT</t>
+  </si>
+  <si>
+    <t>MOV</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Opp</t>
+  </si>
+  <si>
+    <t>Jump</t>
+  </si>
+  <si>
+    <t>Move</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>LOG</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Instruction Layout</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="8"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1010</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="6"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1001</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1011</t>
+    </r>
+  </si>
+  <si>
+    <t>Param 1</t>
+  </si>
+  <si>
+    <t>Param 2</t>
+  </si>
+  <si>
+    <t>Param 3</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>A? reg(B) -&gt; PC</t>
+  </si>
+  <si>
+    <t>reg(B) -&gt; PC, PC -&gt; SRR</t>
+  </si>
+  <si>
+    <t>SRR -&gt; PC</t>
+  </si>
+  <si>
+    <t>reg(A) + reg(B) -&gt; reg(C)</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg(A) - reg(B) -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg(B) # reg(C) -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">mem(0…AB) -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">mem(reg(A) + reg(B)) -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t>reg(C) -&gt; mem(0…AB)</t>
+  </si>
+  <si>
+    <t>reg(C) -&gt; mem(reg(A) + reg(B))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg(C) -&gt; OUT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg(A) -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC -&gt; reg(C) </t>
+  </si>
+  <si>
+    <t>Reg of first number</t>
+  </si>
+  <si>
+    <t>Reg of second number</t>
+  </si>
+  <si>
+    <t>Reg of result</t>
+  </si>
+  <si>
+    <t>Reg of first operand</t>
+  </si>
+  <si>
+    <t>Reg of second operand and result</t>
+  </si>
+  <si>
+    <t>Logic operation (1.)</t>
+  </si>
+  <si>
+    <t>Jump condition (2.)</t>
+  </si>
+  <si>
+    <t>Reg of jump location</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>HLT</t>
+  </si>
+  <si>
+    <t>Misc</t>
+  </si>
+  <si>
+    <t>0 -&gt; CLK</t>
+  </si>
+  <si>
+    <t>Memory location of data</t>
+  </si>
+  <si>
+    <t>Memory location start</t>
+  </si>
+  <si>
+    <t>Memory location dist</t>
+  </si>
+  <si>
+    <t>Reg of data</t>
+  </si>
+  <si>
+    <t>Reg of input</t>
+  </si>
+  <si>
+    <t>Reg of output</t>
+  </si>
+  <si>
+    <t>Reg of source</t>
+  </si>
+  <si>
+    <t>Reg of address</t>
+  </si>
+  <si>
+    <t># of CLK cycles</t>
+  </si>
+  <si>
+    <t>Cycle 1</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -48,13 +346,65 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -69,8 +419,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,9 +782,471 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F4D1BD-2D10-406C-A85F-C78205C3BCE4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="3"/>
+    <col min="2" max="3" width="9.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="24.140625" customWidth="1"/>
+    <col min="10" max="10" width="23.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.42578125" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="4"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E6" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" t="s">
+        <v>80</v>
+      </c>
+      <c r="M6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s">
+        <v>60</v>
+      </c>
+      <c r="J7" t="s">
+        <v>61</v>
+      </c>
+      <c r="K7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E8" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E9" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" t="s">
+        <v>63</v>
+      </c>
+      <c r="K9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" t="s">
+        <v>72</v>
+      </c>
+      <c r="K13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J14" t="s">
+        <v>74</v>
+      </c>
+      <c r="K14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" t="s">
+        <v>72</v>
+      </c>
+      <c r="K15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I16" t="s">
+        <v>73</v>
+      </c>
+      <c r="J16" t="s">
+        <v>74</v>
+      </c>
+      <c r="K16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" t="s">
+        <v>68</v>
+      </c>
+      <c r="J17" t="s">
+        <v>68</v>
+      </c>
+      <c r="K17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" t="s">
+        <v>68</v>
+      </c>
+      <c r="J18" t="s">
+        <v>68</v>
+      </c>
+      <c r="K18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I19" t="s">
+        <v>78</v>
+      </c>
+      <c r="J19" t="s">
+        <v>68</v>
+      </c>
+      <c r="K19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I20" t="s">
+        <v>68</v>
+      </c>
+      <c r="J20" t="s">
+        <v>68</v>
+      </c>
+      <c r="K20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I21" t="s">
+        <v>68</v>
+      </c>
+      <c r="J21" t="s">
+        <v>68</v>
+      </c>
+      <c r="K21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BC93FB-232C-47E9-B1EF-E091B3D3959E}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
made datapath connections in core
</commit_message>
<xml_diff>
--- a/ISA.xlsx
+++ b/ISA.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,14 +10,13 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A7EAE0-63CE-4B6E-BD7D-50AC16A1E5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="Control signals" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -430,9 +429,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -448,6 +444,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -797,46 +796,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="11"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="s">
@@ -848,13 +847,13 @@
       <c r="H6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="6" t="s">
         <v>41</v>
       </c>
       <c r="L6" t="s">

</xml_diff>

<commit_message>
Added MOV in CU
</commit_message>
<xml_diff>
--- a/ISA.xlsx
+++ b/ISA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malco\CPUproj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF39A6A-0D89-4664-A1BF-34691C69C51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E36E2BE-F6B9-46A1-8AC3-432BAEA9752E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
+    <workbookView xWindow="3720" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{B5A1CD67-6CBA-4461-AF5A-E906021A4A2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
   <si>
     <t>Op Code</t>
   </si>
@@ -252,9 +252,6 @@
     <t xml:space="preserve">reg(A) -&gt; reg(C) </t>
   </si>
   <si>
-    <t xml:space="preserve">PC -&gt; reg(C) </t>
-  </si>
-  <si>
     <t>Reg of first number</t>
   </si>
   <si>
@@ -288,9 +285,6 @@
     <t>Misc</t>
   </si>
   <si>
-    <t>0 -&gt; CLK</t>
-  </si>
-  <si>
     <t>Memory location of data</t>
   </si>
   <si>
@@ -312,9 +306,6 @@
     <t>Reg of source</t>
   </si>
   <si>
-    <t>Reg of address</t>
-  </si>
-  <si>
     <t># of CLK cycles</t>
   </si>
   <si>
@@ -327,17 +318,17 @@
     <t>Module</t>
   </si>
   <si>
-    <t>LEA</t>
-  </si>
-  <si>
     <t xml:space="preserve">reg(C) # reg(B) -&gt; reg(B) </t>
+  </si>
+  <si>
+    <t>1 -&gt; CLK</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -369,6 +360,12 @@
     <font>
       <sz val="11"/>
       <color theme="6"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -857,10 +854,10 @@
         <v>41</v>
       </c>
       <c r="L6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="M6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -877,13 +874,13 @@
         <v>48</v>
       </c>
       <c r="I7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7" t="s">
         <v>58</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>59</v>
-      </c>
-      <c r="K7" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -900,13 +897,13 @@
         <v>49</v>
       </c>
       <c r="I8" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" t="s">
         <v>58</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>59</v>
-      </c>
-      <c r="K8" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -920,16 +917,16 @@
         <v>31</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
+        <v>60</v>
+      </c>
+      <c r="K9" t="s">
         <v>61</v>
-      </c>
-      <c r="K9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -946,13 +943,13 @@
         <v>45</v>
       </c>
       <c r="I10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J10" t="s">
         <v>64</v>
       </c>
-      <c r="J10" t="s">
-        <v>65</v>
-      </c>
       <c r="K10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -969,13 +966,13 @@
         <v>46</v>
       </c>
       <c r="I11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -992,13 +989,13 @@
         <v>47</v>
       </c>
       <c r="I12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1015,13 +1012,13 @@
         <v>50</v>
       </c>
       <c r="I13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -1038,13 +1035,13 @@
         <v>51</v>
       </c>
       <c r="I14" t="s">
+        <v>69</v>
+      </c>
+      <c r="J14" t="s">
+        <v>70</v>
+      </c>
+      <c r="K14" t="s">
         <v>71</v>
-      </c>
-      <c r="J14" t="s">
-        <v>72</v>
-      </c>
-      <c r="K14" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -1061,13 +1058,13 @@
         <v>52</v>
       </c>
       <c r="I15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -1084,13 +1081,13 @@
         <v>53</v>
       </c>
       <c r="I16" t="s">
+        <v>69</v>
+      </c>
+      <c r="J16" t="s">
+        <v>70</v>
+      </c>
+      <c r="K16" t="s">
         <v>71</v>
-      </c>
-      <c r="J16" t="s">
-        <v>72</v>
-      </c>
-      <c r="K16" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="17" spans="5:11" x14ac:dyDescent="0.25">
@@ -1107,13 +1104,13 @@
         <v>54</v>
       </c>
       <c r="I17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="5:11" x14ac:dyDescent="0.25">
@@ -1130,13 +1127,13 @@
         <v>55</v>
       </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="5:11" x14ac:dyDescent="0.25">
@@ -1153,13 +1150,13 @@
         <v>56</v>
       </c>
       <c r="I19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="5:11" x14ac:dyDescent="0.25">
@@ -1167,22 +1164,22 @@
         <v>14</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="I20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K20" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="5:11" x14ac:dyDescent="0.25">
@@ -1190,23 +1187,9 @@
         <v>15</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I21" t="s">
-        <v>66</v>
-      </c>
-      <c r="J21" t="s">
-        <v>66</v>
-      </c>
-      <c r="K21" t="s">
-        <v>66</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="G21" s="1"/>
     </row>
     <row r="22" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E22" s="3" t="s">
@@ -1222,6 +1205,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1236,13 +1220,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B1" t="s">
         <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>